<commit_message>
update rekap absen dan nilai
</commit_message>
<xml_diff>
--- a/Rekap Absen dan Nilai 2025-2026.xlsx
+++ b/Rekap Absen dan Nilai 2025-2026.xlsx
@@ -5,15 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="KELAS 11" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="KELAS 10" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="XII IPS" sheetId="3" state="hidden" r:id="rId4"/>
+    <sheet name="KELAS 11" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="KELAS 10" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="XII IPS" sheetId="3" state="hidden" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'KELAS 10'!$A$11:$L$129</definedName>
@@ -4329,16 +4329,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy\ h:mm"/>
-    <numFmt numFmtId="167" formatCode="General"/>
-    <numFmt numFmtId="168" formatCode="0"/>
-    <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="0."/>
-    <numFmt numFmtId="171" formatCode="0%"/>
-    <numFmt numFmtId="172" formatCode="_([$Rp-421]* #,##0_);_([$Rp-421]* \(#,##0\);_([$Rp-421]* \-_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="0."/>
+    <numFmt numFmtId="170" formatCode="0%"/>
+    <numFmt numFmtId="171" formatCode="_([$Rp-421]* #,##0_);_([$Rp-421]* \(#,##0\);_([$Rp-421]* \-_);_(@_)"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -4878,7 +4877,7 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -5067,15 +5066,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5123,7 +5122,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5155,7 +5154,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5163,11 +5162,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="22" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5215,7 +5214,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5311,11 +5310,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5415,7 +5414,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5431,7 +5430,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5443,7 +5442,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5459,7 +5458,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5523,11 +5522,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="47" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="47" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="48" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="48" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5547,11 +5546,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -5623,7 +5622,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="47" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="47" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5635,7 +5634,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -5655,7 +5654,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -5663,11 +5662,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -5691,11 +5690,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="45" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="45" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -5743,7 +5742,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5751,6 +5750,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5758,7 +5758,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF000000"/>
-          <bgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5766,6 +5766,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF00A933"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5773,6 +5774,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF81D41A"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5780,6 +5782,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFBF819E"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5787,6 +5790,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFDEE6EF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5794,6 +5798,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFA6A6"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5801,6 +5806,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFD428"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5900,10 +5906,10 @@
       <xdr:rowOff>65160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>3240</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>402480</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -5913,9 +5919,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="1170000"/>
-          <a:ext cx="14657400" cy="28800"/>
+          <a:ext cx="5119560" cy="29160"/>
           <a:chOff x="35280" y="1170000"/>
-          <a:chExt cx="14657400" cy="28800"/>
+          <a:chExt cx="5119560" cy="29160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -5925,8 +5931,8 @@
         </xdr:nvCxnSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="39240" y="1188000"/>
-            <a:ext cx="14653800" cy="11160"/>
+            <a:off x="36720" y="1188000"/>
+            <a:ext cx="5118480" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -5947,7 +5953,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="1170000"/>
-            <a:ext cx="14653800" cy="11160"/>
+            <a:ext cx="5118480" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -5972,9 +5978,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>738360</xdr:colOff>
+      <xdr:colOff>738000</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>113400</xdr:rowOff>
+      <xdr:rowOff>113040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -5989,11 +5995,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="57240"/>
-          <a:ext cx="1070280" cy="818280"/>
+          <a:ext cx="1069920" cy="817920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6010,9 +6017,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>738360</xdr:colOff>
+      <xdr:colOff>738000</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>132480</xdr:rowOff>
+      <xdr:rowOff>132120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6027,11 +6034,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="8439120"/>
-          <a:ext cx="1070280" cy="818280"/>
+          <a:ext cx="1069920" cy="817920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6048,9 +6056,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>738360</xdr:colOff>
+      <xdr:colOff>738000</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>132480</xdr:rowOff>
+      <xdr:rowOff>132120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6065,11 +6073,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="8439120"/>
-          <a:ext cx="1070280" cy="818280"/>
+          <a:ext cx="1069920" cy="817920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6085,10 +6094,10 @@
       <xdr:rowOff>65160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>3240</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>402480</xdr:colOff>
       <xdr:row>55</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6098,9 +6107,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="9771120"/>
-          <a:ext cx="14657400" cy="28800"/>
+          <a:ext cx="5119560" cy="29160"/>
           <a:chOff x="35280" y="9771120"/>
-          <a:chExt cx="14657400" cy="28800"/>
+          <a:chExt cx="5119560" cy="29160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6110,8 +6119,8 @@
         </xdr:nvCxnSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="39240" y="9789120"/>
-            <a:ext cx="14653800" cy="11160"/>
+            <a:off x="36720" y="9789120"/>
+            <a:ext cx="5118480" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6132,7 +6141,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="9771120"/>
-            <a:ext cx="14653800" cy="11160"/>
+            <a:ext cx="5118480" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6157,9 +6166,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>738360</xdr:colOff>
+      <xdr:colOff>738000</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>126000</xdr:rowOff>
+      <xdr:rowOff>125640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6174,11 +6183,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="8667720"/>
-          <a:ext cx="1070280" cy="821520"/>
+          <a:ext cx="1069920" cy="821160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6194,10 +6204,10 @@
       <xdr:rowOff>65160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>3240</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>402480</xdr:colOff>
       <xdr:row>114</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6207,9 +6217,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="20096280"/>
-          <a:ext cx="14657400" cy="28800"/>
+          <a:ext cx="5119560" cy="29160"/>
           <a:chOff x="35280" y="20096280"/>
-          <a:chExt cx="14657400" cy="28800"/>
+          <a:chExt cx="5119560" cy="29160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6219,8 +6229,8 @@
         </xdr:nvCxnSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="39240" y="20114280"/>
-            <a:ext cx="14653800" cy="11160"/>
+            <a:off x="36720" y="20114280"/>
+            <a:ext cx="5118480" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6241,7 +6251,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="20096280"/>
-            <a:ext cx="14653800" cy="11160"/>
+            <a:ext cx="5118480" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6266,9 +6276,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>741960</xdr:colOff>
+      <xdr:colOff>741600</xdr:colOff>
       <xdr:row>112</xdr:row>
-      <xdr:rowOff>107640</xdr:rowOff>
+      <xdr:rowOff>107280</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -6278,7 +6288,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4320" y="18977760"/>
-          <a:ext cx="1070280" cy="817920"/>
+          <a:ext cx="1069920" cy="817560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6309,15 +6319,19 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-US" sz="1800" spc="-1" strike="noStrike">
+            <a:rPr b="0" lang="en-US" sz="1800" strike="noStrike" u="none">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
+              <a:effectLst/>
+              <a:uFillTx/>
               <a:latin typeface="Times New Roman"/>
             </a:rPr>
             <a:t>Cxz </a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1800" spc="-1" strike="noStrike">
+          <a:endParaRPr b="0" lang="en-US" sz="1800" strike="noStrike" u="none">
+            <a:effectLst/>
+            <a:uFillTx/>
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -6339,9 +6353,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>360</xdr:colOff>
+      <xdr:colOff>720</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6351,9 +6365,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="1112760"/>
-          <a:ext cx="2832120" cy="28800"/>
+          <a:ext cx="2832480" cy="29160"/>
           <a:chOff x="35280" y="1112760"/>
-          <a:chExt cx="2832120" cy="28800"/>
+          <a:chExt cx="2832480" cy="29160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6364,7 +6378,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36360" y="1130760"/>
-            <a:ext cx="2831400" cy="11160"/>
+            <a:ext cx="2831760" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6385,7 +6399,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="1112760"/>
-            <a:ext cx="2831400" cy="11160"/>
+            <a:ext cx="2831760" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6410,9 +6424,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>751680</xdr:colOff>
+      <xdr:colOff>751320</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>24480</xdr:rowOff>
+      <xdr:rowOff>24120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6427,11 +6441,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="57240"/>
-          <a:ext cx="1069560" cy="824400"/>
+          <a:ext cx="1069200" cy="824040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6448,9 +6463,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>360</xdr:colOff>
+      <xdr:colOff>720</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6460,9 +6475,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="12190320"/>
-          <a:ext cx="2832120" cy="28800"/>
+          <a:ext cx="2832480" cy="29160"/>
           <a:chOff x="35280" y="12190320"/>
-          <a:chExt cx="2832120" cy="28800"/>
+          <a:chExt cx="2832480" cy="29160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6473,7 +6488,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36360" y="12208320"/>
-            <a:ext cx="2831400" cy="11160"/>
+            <a:ext cx="2831760" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6494,7 +6509,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="12190320"/>
-            <a:ext cx="2831400" cy="11160"/>
+            <a:ext cx="2831760" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6519,9 +6534,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>751680</xdr:colOff>
+      <xdr:colOff>751320</xdr:colOff>
       <xdr:row>72</xdr:row>
-      <xdr:rowOff>24480</xdr:rowOff>
+      <xdr:rowOff>24120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6536,11 +6551,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="11134800"/>
-          <a:ext cx="1069560" cy="824400"/>
+          <a:ext cx="1069200" cy="824040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6557,9 +6573,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>360</xdr:colOff>
+      <xdr:colOff>720</xdr:colOff>
       <xdr:row>140</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>94320</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6569,9 +6585,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="23296680"/>
-          <a:ext cx="2832120" cy="28800"/>
+          <a:ext cx="2832480" cy="29160"/>
           <a:chOff x="35280" y="23296680"/>
-          <a:chExt cx="2832120" cy="28800"/>
+          <a:chExt cx="2832480" cy="29160"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6582,7 +6598,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36360" y="23314680"/>
-            <a:ext cx="2831400" cy="11160"/>
+            <a:ext cx="2831760" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6603,7 +6619,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="23296680"/>
-            <a:ext cx="2831400" cy="11160"/>
+            <a:ext cx="2831760" cy="11520"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6628,9 +6644,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>751680</xdr:colOff>
+      <xdr:colOff>751320</xdr:colOff>
       <xdr:row>139</xdr:row>
-      <xdr:rowOff>24480</xdr:rowOff>
+      <xdr:rowOff>24120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6645,11 +6661,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="22240800"/>
-          <a:ext cx="1069560" cy="824760"/>
+          <a:ext cx="1069200" cy="824400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6671,9 +6688,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>46080</xdr:colOff>
+      <xdr:colOff>45720</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>150840</xdr:rowOff>
+      <xdr:rowOff>150480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6687,11 +6704,12 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="359640" y="238320"/>
-          <a:ext cx="795240" cy="922320"/>
+          <a:ext cx="794880" cy="921960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -6735,13 +6753,119 @@
 </externalLink>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AH1048576"/>
-  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="13.5" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.72"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="2" min="2" style="1" width="11.51"/>
@@ -6756,22 +6880,22 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="12" min="12" style="2" width="14.52"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="13" min="13" style="2" width="11.51"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="14" min="14" style="4" width="6.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="5" width="9.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="5.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="5.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="8.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="10.56"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="11.51"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="22" min="22" style="5" width="11.51"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="11.51"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="24" min="24" style="2" width="11.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="13.49"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="27" min="26" style="1" width="11.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="11.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="6" width="6.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="6.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="2" width="8.11"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="15" min="15" style="5" width="9.58"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="16" min="16" style="2" width="5.71"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="17" min="17" style="1" width="5.71"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="18" min="18" style="1" width="8.29"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="19" min="19" style="1" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="20" min="20" style="1" width="10.56"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="21" min="21" style="1" width="11.51"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="22" min="22" style="5" width="11.51"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="23" min="23" style="1" width="11.51"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="24" min="24" style="2" width="11.51"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="25" min="25" style="1" width="13.49"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="27" min="26" style="1" width="11.51"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="28" min="28" style="1" width="11.24"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="29" min="29" style="6" width="6.61"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="30" min="30" style="1" width="6.96"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="31" min="31" style="2" width="8.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="9.62"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="33" style="2" width="11.51"/>
   </cols>
@@ -18002,7 +18126,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AJ201"/>
-  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="77" width="4.52"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="2" min="2" style="77" width="11.51"/>
@@ -30490,7 +30614,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:XFD283"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="139" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="139" width="11.44"/>

</xml_diff>

<commit_message>
update readku dan rekap nilai
</commit_message>
<xml_diff>
--- a/Rekap Absen dan Nilai 2025-2026.xlsx
+++ b/Rekap Absen dan Nilai 2025-2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="KELAS 11" sheetId="1" state="visible" r:id="rId3"/>
@@ -5956,9 +5956,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>4320</xdr:colOff>
+      <xdr:colOff>4680</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>98640</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -5968,9 +5968,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="1170000"/>
-          <a:ext cx="5634360" cy="33480"/>
+          <a:ext cx="5634720" cy="33840"/>
           <a:chOff x="35280" y="1170000"/>
-          <a:chExt cx="5634360" cy="33480"/>
+          <a:chExt cx="5634720" cy="33840"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -5981,7 +5981,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36720" y="1188000"/>
-            <a:ext cx="5633280" cy="15840"/>
+            <a:ext cx="5633640" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6002,7 +6002,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="1170000"/>
-            <a:ext cx="5632920" cy="15840"/>
+            <a:ext cx="5633280" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6027,9 +6027,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>733680</xdr:colOff>
+      <xdr:colOff>733320</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>108720</xdr:rowOff>
+      <xdr:rowOff>108360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6044,7 +6044,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="57240"/>
-          <a:ext cx="1098720" cy="813600"/>
+          <a:ext cx="1098360" cy="813240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6066,9 +6066,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>733680</xdr:colOff>
+      <xdr:colOff>733320</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>127800</xdr:rowOff>
+      <xdr:rowOff>127440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6083,7 +6083,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="8439840"/>
-          <a:ext cx="1098720" cy="813600"/>
+          <a:ext cx="1098360" cy="813240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6105,9 +6105,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>733680</xdr:colOff>
+      <xdr:colOff>733320</xdr:colOff>
       <xdr:row>52</xdr:row>
-      <xdr:rowOff>127800</xdr:rowOff>
+      <xdr:rowOff>127440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6122,7 +6122,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="8439840"/>
-          <a:ext cx="1098720" cy="813600"/>
+          <a:ext cx="1098360" cy="813240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6144,9 +6144,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>4320</xdr:colOff>
+      <xdr:colOff>4680</xdr:colOff>
       <xdr:row>55</xdr:row>
-      <xdr:rowOff>98640</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6156,9 +6156,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="9771840"/>
-          <a:ext cx="5634360" cy="33480"/>
+          <a:ext cx="5634720" cy="33840"/>
           <a:chOff x="35280" y="9771840"/>
-          <a:chExt cx="5634360" cy="33480"/>
+          <a:chExt cx="5634720" cy="33840"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6169,7 +6169,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36720" y="9789840"/>
-            <a:ext cx="5633280" cy="15840"/>
+            <a:ext cx="5633640" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6190,7 +6190,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="9771840"/>
-            <a:ext cx="5632920" cy="15840"/>
+            <a:ext cx="5633280" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6215,9 +6215,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>733680</xdr:colOff>
+      <xdr:colOff>733320</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>121680</xdr:rowOff>
+      <xdr:rowOff>121320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6232,7 +6232,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="8668440"/>
-          <a:ext cx="1098720" cy="816840"/>
+          <a:ext cx="1098360" cy="816480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6254,9 +6254,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>4320</xdr:colOff>
+      <xdr:colOff>4680</xdr:colOff>
       <xdr:row>114</xdr:row>
-      <xdr:rowOff>98640</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6266,9 +6266,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="20097000"/>
-          <a:ext cx="5634360" cy="33480"/>
+          <a:ext cx="5634720" cy="33840"/>
           <a:chOff x="35280" y="20097000"/>
-          <a:chExt cx="5634360" cy="33480"/>
+          <a:chExt cx="5634720" cy="33840"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6279,7 +6279,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36720" y="20115000"/>
-            <a:ext cx="5633280" cy="15840"/>
+            <a:ext cx="5633640" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6300,7 +6300,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="20097000"/>
-            <a:ext cx="5632920" cy="15840"/>
+            <a:ext cx="5633280" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6325,9 +6325,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>737280</xdr:colOff>
+      <xdr:colOff>736920</xdr:colOff>
       <xdr:row>112</xdr:row>
-      <xdr:rowOff>102600</xdr:rowOff>
+      <xdr:rowOff>102240</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -6337,7 +6337,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4320" y="18978120"/>
-          <a:ext cx="1098720" cy="813240"/>
+          <a:ext cx="1098360" cy="812880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6403,9 +6403,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>5040</xdr:colOff>
+      <xdr:colOff>5400</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>98640</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6415,9 +6415,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="1112760"/>
-          <a:ext cx="3120120" cy="33480"/>
+          <a:ext cx="3120480" cy="33840"/>
           <a:chOff x="35280" y="1112760"/>
-          <a:chExt cx="3120120" cy="33480"/>
+          <a:chExt cx="3120480" cy="33840"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6428,7 +6428,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36360" y="1130760"/>
-            <a:ext cx="3119400" cy="15840"/>
+            <a:ext cx="3119760" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6449,7 +6449,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="1112760"/>
-            <a:ext cx="3119040" cy="15840"/>
+            <a:ext cx="3119400" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6474,9 +6474,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>747000</xdr:colOff>
+      <xdr:colOff>746640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>19800</xdr:rowOff>
+      <xdr:rowOff>19440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6491,7 +6491,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="57240"/>
-          <a:ext cx="1096200" cy="819720"/>
+          <a:ext cx="1095840" cy="819360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6513,9 +6513,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>5040</xdr:colOff>
+      <xdr:colOff>5400</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>98640</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6525,9 +6525,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="12190320"/>
-          <a:ext cx="3120120" cy="33480"/>
+          <a:ext cx="3120480" cy="33840"/>
           <a:chOff x="35280" y="12190320"/>
-          <a:chExt cx="3120120" cy="33480"/>
+          <a:chExt cx="3120480" cy="33840"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6538,7 +6538,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36360" y="12208320"/>
-            <a:ext cx="3119400" cy="15840"/>
+            <a:ext cx="3119760" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6559,7 +6559,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="12190320"/>
-            <a:ext cx="3119040" cy="15840"/>
+            <a:ext cx="3119400" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6584,9 +6584,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>747000</xdr:colOff>
+      <xdr:colOff>746640</xdr:colOff>
       <xdr:row>72</xdr:row>
-      <xdr:rowOff>19800</xdr:rowOff>
+      <xdr:rowOff>19440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6601,7 +6601,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="11134800"/>
-          <a:ext cx="1096200" cy="819720"/>
+          <a:ext cx="1095840" cy="819360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6623,9 +6623,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>5040</xdr:colOff>
+      <xdr:colOff>5400</xdr:colOff>
       <xdr:row>140</xdr:row>
-      <xdr:rowOff>98640</xdr:rowOff>
+      <xdr:rowOff>99000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -6635,9 +6635,9 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="35280" y="23296680"/>
-          <a:ext cx="3120120" cy="33480"/>
+          <a:ext cx="3120480" cy="33840"/>
           <a:chOff x="35280" y="23296680"/>
-          <a:chExt cx="3120120" cy="33480"/>
+          <a:chExt cx="3120480" cy="33840"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:cxnSp>
@@ -6648,7 +6648,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="36360" y="23314680"/>
-            <a:ext cx="3119400" cy="15840"/>
+            <a:ext cx="3119760" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6669,7 +6669,7 @@
         <xdr:spPr>
           <a:xfrm>
             <a:off x="35280" y="23296680"/>
-            <a:ext cx="3119040" cy="15840"/>
+            <a:ext cx="3119400" cy="16200"/>
           </a:xfrm>
           <a:prstGeom prst="straightConnector1">
             <a:avLst/>
@@ -6694,9 +6694,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>747000</xdr:colOff>
+      <xdr:colOff>746640</xdr:colOff>
       <xdr:row>139</xdr:row>
-      <xdr:rowOff>19800</xdr:rowOff>
+      <xdr:rowOff>19440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6711,7 +6711,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="720" y="22240800"/>
-          <a:ext cx="1096200" cy="820080"/>
+          <a:ext cx="1095840" cy="819720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6738,9 +6738,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>41400</xdr:colOff>
+      <xdr:colOff>41040</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>146160</xdr:rowOff>
+      <xdr:rowOff>145800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6754,7 +6754,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="389520" y="238320"/>
-          <a:ext cx="870480" cy="917640"/>
+          <a:ext cx="870120" cy="917280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8715,7 +8715,7 @@
       </c>
       <c r="AJ26" s="31"/>
       <c r="AK26" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9961,7 +9961,7 @@
       </c>
       <c r="AJ38" s="31"/>
       <c r="AK38" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>